<commit_message>
feat: home v2 重打 (2,117 菜) + 两 zone review 样本
- home v2-promptfix 全量重打: 43 批 × 50/批, 16 并发 × 3 轮, 0 failed
- 两 zone 各 50 条 review_sample (md + xlsx, seed=42 可复现) 待人工 review
- 至此两 zone 13,240 菜全部 v2-promptfix, 数据 + 打标阶段告一段落
- ROADMAP 当前状态 + DECISIONS D-031 执行进度同步更新

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/shenzhen-bay/review_sample.xlsx
+++ b/data/shenzhen-bay/review_sample.xlsx
@@ -431,8 +431,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
-    <col width="31" customWidth="1" min="2" max="2"/>
-    <col width="31" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
     <col width="7" customWidth="1" min="4" max="4"/>
     <col width="9" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
@@ -521,51 +521,47 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>d_098_080</t>
+          <t>d_208_078</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>汕头达濠鱼丸汤面</t>
+          <t>蒜蓉炒红薯叶（不含米饭）</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>汕头达濠鱼丸汤面</t>
+          <t>蒜蓉炒红薯叶</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>20.8</v>
+        <v>32</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>潮汕</t>
+          <t>湘菜</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>纯素</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>煮</t>
+          <t>炒</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I2" t="n">
-        <v>0.1</v>
+        <v>0.95</v>
       </c>
       <c r="J2" t="n">
-        <v>15</v>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>0</v>
       </c>
@@ -575,25 +571,25 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>d_015_044</t>
+          <t>d_028_045</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>爆浆红糖糍粑</t>
+          <t>招牌普宁肠粉++香浓豆浆++杭州小笼包 6 个</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>爆浆红糖糍粑</t>
+          <t>普宁肠粉+豆浆+杭州小笼包 6 个</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>2.6</v>
+        <v>33.8</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>小吃</t>
+          <t>粤菜</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -603,19 +599,23 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>油炸</t>
+          <t>蒸</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="J3" t="n">
-        <v>2</v>
-      </c>
-      <c r="K3" t="inlineStr"/>
+        <v>20</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="L3" t="n">
         <v>0</v>
       </c>
@@ -625,49 +625,49 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>d_004_011</t>
+          <t>d_007_030</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>【❤️宠粉福利】剁椒萝卜干（每单限一份，多点不送）</t>
+          <t>盐焗花螺</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>剁椒萝卜干</t>
+          <t>盐焗花螺</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.5</v>
+        <v>108</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>湘菜</t>
+          <t>粤菜</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>纯素</t>
+          <t>海鲜</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>凉拌</t>
+          <t>烤</t>
         </is>
       </c>
       <c r="H4" t="n">
         <v>2</v>
       </c>
       <c r="I4" t="n">
-        <v>0.9</v>
+        <v>0.05</v>
       </c>
       <c r="J4" t="n">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr"/>
@@ -675,25 +675,25 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>d_118_029</t>
+          <t>d_087_018</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>酸辣河粉</t>
+          <t>鸳鸯大小骨</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>酸辣河粉</t>
+          <t>鸳鸯大小骨粉</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>16.8</v>
+        <v>31</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>川菜</t>
+          <t>湘菜</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -713,11 +713,15 @@
         <v>0.05</v>
       </c>
       <c r="J5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K5" t="inlineStr"/>
+        <v>25</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="L5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
@@ -725,51 +729,47 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>d_039_051</t>
+          <t>d_075_068</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>鸡蛋肉丝炒鸳鸯粉</t>
+          <t>莲子猪心汤</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>鸡蛋肉丝炒鸳鸯粉</t>
+          <t>莲子猪心汤</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>18</v>
+        <v>16.9</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>粤菜</t>
+          <t>汤粥</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>汤</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>炒</t>
+          <t>炖</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I6" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="J6" t="n">
         <v>15</v>
       </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+      <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
         <v>0</v>
       </c>
@@ -779,45 +779,45 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>d_031_021</t>
+          <t>d_069_051</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>天妇罗蟹柳(5 个)</t>
+          <t>白切鸡整只（不配饭</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>天妇罗蟹柳</t>
+          <t>白切鸡整只</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>18</v>
+        <v>88</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>日式</t>
+          <t>粤菜</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>海鲜</t>
+          <t>白肉</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>油炸</t>
+          <t>煮</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
@@ -829,30 +829,30 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>d_028_049</t>
+          <t>d_042_010</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>加老家菜脯粒</t>
+          <t>牛肉炒饭</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>加老家菜脯粒</t>
+          <t>牛肉炒饭</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2.8</v>
+        <v>28</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>潮汕</t>
+          <t>粤菜</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>纯素</t>
+          <t>主食</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -861,15 +861,19 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I8" t="n">
-        <v>0.7</v>
+        <v>0.1</v>
       </c>
       <c r="J8" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" t="inlineStr"/>
+        <v>20</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="L8" t="n">
         <v>0</v>
       </c>
@@ -879,25 +883,25 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>d_018_062</t>
+          <t>d_026_046</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>爆炒酸辣土豆丝（不配饭）</t>
+          <t>锡纸盒烧金针菇</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>爆炒酸辣土豆丝</t>
+          <t>锡纸盒烧金针菇</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>15.8</v>
+        <v>28</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>湘菜</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -907,7 +911,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>炒</t>
+          <t>烤</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -917,11 +921,11 @@
         <v>0.9</v>
       </c>
       <c r="J9" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
@@ -929,49 +933,53 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>d_117_010</t>
+          <t>d_223_022</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>蒸面</t>
+          <t>特色肉肠拌菜套餐</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>蒸面</t>
+          <t>特色肉肠拌菜套餐</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>14</v>
+        <v>25.8</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>粤菜</t>
+          <t>川菜</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>红肉</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>蒸</t>
+          <t>凉拌</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I10" t="n">
-        <v>0.05</v>
+        <v>0.3</v>
       </c>
       <c r="J10" t="n">
-        <v>8</v>
-      </c>
-      <c r="K10" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="L10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
@@ -979,49 +987,49 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>d_014_042</t>
+          <t>d_176_065</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>包浆豆腐（1）</t>
+          <t>手工辣椒酱小盒（1 个饭限 1 份酱料，多点不送）</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>包浆豆腐</t>
+          <t>手工辣椒酱</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>26.9</v>
+        <v>0.5</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>小吃</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>豆制品</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>烤</t>
+          <t>生</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="J11" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
@@ -1029,25 +1037,25 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>d_106_034</t>
+          <t>d_022_057</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>【双人】皮蛋瘦肉砂锅粥+茂名捞粉套餐</t>
+          <t>☀️爆汁韭黄牛肉水饺</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>皮蛋瘦肉砂锅粥茂名捞粉双人套餐</t>
+          <t>爆汁韭黄牛肉水饺</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>34.7</v>
+        <v>33</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>粤菜</t>
+          <t>西北</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -1064,10 +1072,10 @@
         <v>2</v>
       </c>
       <c r="I12" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J12" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -1083,21 +1091,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>d_118_022</t>
+          <t>d_192_005</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>加排骨</t>
+          <t>工作单人餐 A</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>加排骨</t>
+          <t>工作单人餐A</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>11.1</v>
+        <v>46</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -1111,21 +1119,25 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>炖</t>
+          <t>炒</t>
         </is>
       </c>
       <c r="H13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I13" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="J13" t="n">
-        <v>15</v>
-      </c>
-      <c r="K13" t="inlineStr"/>
+        <v>25</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="L13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
@@ -1133,45 +1145,45 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>d_086_013</t>
+          <t>d_132_040</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>板烧鸡腿堡套餐</t>
+          <t>螺蛳粉+1*加多宝</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>板烧鸡腿堡套餐</t>
+          <t>螺蛳粉</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>41.5</v>
+        <v>23.5</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>快餐</t>
+          <t>小吃</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>白肉</t>
+          <t>主食</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>煎</t>
+          <t>煮</t>
         </is>
       </c>
       <c r="H14" t="n">
         <v>4</v>
       </c>
       <c r="I14" t="n">
-        <v>0.08</v>
+        <v>0.15</v>
       </c>
       <c r="J14" t="n">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -1179,7 +1191,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
@@ -1187,21 +1199,21 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>d_013_001</t>
+          <t>d_008_058</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>【新店福利】烤马可波罗肠</t>
+          <t>面筋#坚持纯手工</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>烤马可波罗肠</t>
+          <t>面筋</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>15</v>
+        <v>3.7</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -1210,7 +1222,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>红肉</t>
+          <t>主食</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1225,11 +1237,11 @@
         <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
@@ -1237,53 +1249,49 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>d_091_061</t>
+          <t>d_008_026</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>公主王子请下单，套餐 4 种可选（划算实惠）</t>
+          <t>牛肉丸#纯正新鲜</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>公主王子套餐</t>
+          <t>牛肉丸</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>23.9</v>
+        <v>3.4</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>粤菜</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>红肉</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>蒸</t>
+          <t>烤</t>
         </is>
       </c>
       <c r="H16" t="n">
         <v>3</v>
       </c>
       <c r="I16" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J16" t="n">
-        <v>18</v>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="K16" t="inlineStr"/>
       <c r="L16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr"/>
@@ -1291,49 +1299,53 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>d_064_022</t>
+          <t>d_024_033</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>煲粥马蹄（不可单点，需配海鲜粥类）</t>
+          <t>砂锅蟹味棒米线</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>煲粥马蹄</t>
+          <t>砂锅蟹味棒米线</t>
         </is>
       </c>
       <c r="D17" t="n">
+        <v>20</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>小吃</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>主食</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>煮</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>3</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="J17" t="n">
         <v>10</v>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>粤菜</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>纯素</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>煮</t>
-        </is>
-      </c>
-      <c r="H17" t="n">
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
         <v>1</v>
-      </c>
-      <c r="I17" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="J17" t="n">
-        <v>2</v>
-      </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="n">
-        <v>0</v>
       </c>
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr"/>
@@ -1341,30 +1353,30 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>d_005_005</t>
+          <t>d_068_052</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>【邓凯同款】喜笑颜“凯”套餐</t>
+          <t>脆皮香肠 1 根</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>喜笑颜凯套餐</t>
+          <t>脆皮香肠 1 根</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>39.9</v>
+        <v>4.9</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>小吃</t>
+          <t>西式</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>红肉</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1376,14 +1388,14 @@
         <v>5</v>
       </c>
       <c r="I18" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J18" t="n">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr"/>
@@ -1391,49 +1403,53 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>d_004_051</t>
+          <t>d_072_017</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>娃哈哈</t>
+          <t>红油麻辣猪肉小馄饨</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>娃哈哈</t>
+          <t>红油麻辣猪肉小馄饨</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>26.8</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>江浙</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>主食</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>生</t>
+          <t>煮</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="J19" t="n">
+        <v>15</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
         <v>2</v>
-      </c>
-      <c r="K19" t="inlineStr"/>
-      <c r="L19" t="n">
-        <v>0</v>
       </c>
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr"/>
@@ -1441,21 +1457,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>d_013_056</t>
+          <t>d_163_054</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>丹东大黄蚬子</t>
+          <t>褔鼎肉片+卡兹脆鸡排+可乐 300ml</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>丹东大黄蚬子</t>
+          <t>福鼎肉片+卡兹脆鸡排+可乐 300ml</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>98</v>
+        <v>27.9</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1464,22 +1480,22 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>海鲜</t>
+          <t>红肉</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>烤</t>
+          <t>油炸</t>
         </is>
       </c>
       <c r="H20" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="I20" t="n">
         <v>0.05</v>
       </c>
       <c r="J20" t="n">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="n">
@@ -1491,51 +1507,47 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>d_028_012</t>
+          <t>d_195_043</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>双蛋瘦肉肠粉</t>
+          <t>柳州腊肠（1 根）</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>双蛋瘦肉肠粉</t>
+          <t>柳州腊肠 1 根</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>26.8</v>
+        <v>4.9</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>潮汕</t>
+          <t>小吃</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>红肉</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>蒸</t>
+          <t>煎</t>
         </is>
       </c>
       <c r="H21" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I21" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>22</v>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="K21" t="inlineStr"/>
       <c r="L21" t="n">
         <v>0</v>
       </c>
@@ -1545,45 +1557,45 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>d_029_049</t>
+          <t>d_007_055</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>玉米</t>
+          <t>铁板姜汁芥兰牛肉</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>玉米</t>
+          <t>铁板姜汁芥兰牛肉</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>10</v>
+        <v>42</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>粤菜</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>红肉</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>烤</t>
+          <t>炒</t>
         </is>
       </c>
       <c r="H22" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I22" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="J22" t="n">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="n">
@@ -1595,21 +1607,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>d_079_047</t>
+          <t>d_181_048</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>杂菜煲</t>
+          <t>顺德炸酸奶</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>杂菜煲</t>
+          <t>顺德炸酸奶</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1618,22 +1630,22 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>纯素</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>炖</t>
+          <t>油炸</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I23" t="n">
-        <v>0.85</v>
+        <v>0</v>
       </c>
       <c r="J23" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="n">
@@ -1645,45 +1657,45 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>d_092_074</t>
+          <t>d_061_018</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>生炒牛肉</t>
+          <t>鸡生蚝肉</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>生炒牛肉</t>
+          <t>鸡生蚝肉</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>58</v>
+        <v>18</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>粤菜</t>
+          <t>日式</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>红肉</t>
+          <t>白肉</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>炒</t>
+          <t>烤</t>
         </is>
       </c>
       <c r="H24" t="n">
         <v>4</v>
       </c>
       <c r="I24" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>45</v>
+        <v>15</v>
       </c>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="n">
@@ -1695,53 +1707,49 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>d_004_024</t>
+          <t>d_214_014</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>【能量满格】湘式剁椒蛋炒饭 加码自选套餐</t>
+          <t>冻柠乐</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>湘式剁椒蛋炒饭加码自选套餐</t>
+          <t>冻柠乐</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>26.8</v>
+        <v>7</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>湘菜</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>炒</t>
+          <t>生</t>
         </is>
       </c>
       <c r="H25" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I25" t="n">
-        <v>0.15</v>
+        <v>0</v>
       </c>
       <c r="J25" t="n">
-        <v>18</v>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K25" t="inlineStr"/>
       <c r="L25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr"/>
@@ -1749,53 +1757,49 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>d_088_029</t>
+          <t>d_176_058</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>（麻辣牛肉十排骨）汤粉</t>
+          <t>炖足 2 小时..原蛊花旗参炖竹丝鸡汤</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>麻辣牛肉排骨汤粉</t>
+          <t>原盅花旗参炖竹丝鸡汤</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>28.9</v>
+        <v>11.8</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>湘菜</t>
+          <t>粤菜</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>红肉</t>
+          <t>汤</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>煮</t>
+          <t>炖</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I26" t="n">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="J26" t="n">
-        <v>28</v>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr"/>
@@ -1803,49 +1807,53 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>d_025_055</t>
+          <t>d_132_001</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>维他柠檬茶</t>
+          <t>麻辣牛肉粉（汤粉）</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>维他柠檬茶</t>
+          <t>麻辣牛肉粉汤粉</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>7</v>
+        <v>20.5</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>小吃</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>主食</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>生</t>
+          <t>煮</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="J27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="L27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr"/>
@@ -1853,21 +1861,21 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>d_114_010</t>
+          <t>d_069_005</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>斋肠</t>
+          <t>荔枝木烧鹅例牌（不配饭</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>斋肠</t>
+          <t>荔枝木烧鹅例牌(不配饭)</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>6</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1876,22 +1884,22 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>白肉</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>蒸</t>
+          <t>烤</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I28" t="n">
         <v>0</v>
       </c>
       <c r="J28" t="n">
-        <v>4</v>
+        <v>50</v>
       </c>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="n">
@@ -1903,25 +1911,25 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>d_100_016</t>
+          <t>d_142_009</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>【吉祥三宝】紫菜虾米鲜肉小馄饨+老面鲜肉小笼包+龙井茶叶蛋</t>
+          <t>【..招牌】腊味煲仔饭+马蹄椰子鸡汤(小份)单人套餐</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>吉祥三宝（紫菜虾米鲜肉小馄饨+老面鲜肉小笼包+龙井茶叶蛋）</t>
+          <t>腊味煲仔饭+马蹄椰子鸡汤单人套餐 小份</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>28.9</v>
+        <v>53.9</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>江浙</t>
+          <t>粤菜</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -1938,10 +1946,10 @@
         <v>3</v>
       </c>
       <c r="I29" t="n">
-        <v>0.08</v>
+        <v>0.15</v>
       </c>
       <c r="J29" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -1957,51 +1965,47 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>d_112_028</t>
+          <t>d_191_037</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>营养双蛋肠/香滑瘦肉肠随心选套餐+豆浆</t>
+          <t>无糖可口可乐</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>营养双蛋肠/香滑瘦肉肠套餐+豆浆</t>
+          <t>无糖可口可乐</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>18.9</v>
+        <v>5</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>粤菜</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>蒸</t>
+          <t>生</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I30" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>18</v>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" t="n">
         <v>0</v>
       </c>
@@ -2011,53 +2015,49 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>d_086_010</t>
+          <t>d_087_069</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>王牌吃鸡双人随心选</t>
+          <t>辣椒炒肉（直接加粉里）</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>王牌吃鸡双人随心选</t>
+          <t>辣椒炒肉</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>49.9</v>
+        <v>17.8</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>快餐</t>
+          <t>湘菜</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>白肉</t>
+          <t>红肉</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>油炸</t>
+          <t>炒</t>
         </is>
       </c>
       <c r="H31" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I31" t="n">
-        <v>0.03</v>
+        <v>0.3</v>
       </c>
       <c r="J31" t="n">
-        <v>50</v>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="K31" t="inlineStr"/>
       <c r="L31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr"/>
@@ -2065,35 +2065,35 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>d_064_002</t>
+          <t>d_002_059</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>九节虾鲍鱼仔粥（2 人餐）</t>
+          <t>捞汁花甲</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>九节虾鲍鱼仔粥</t>
+          <t>捞汁花甲</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>122.1</v>
+        <v>49</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>粤菜</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>海鲜</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>煮</t>
+          <t>凉拌</t>
         </is>
       </c>
       <c r="H32" t="n">
@@ -2103,15 +2103,11 @@
         <v>0.05</v>
       </c>
       <c r="J32" t="n">
-        <v>60</v>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="K32" t="inlineStr"/>
       <c r="L32" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr"/>
@@ -2119,45 +2115,45 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>d_028_026</t>
+          <t>d_047_049</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>戴记特色腐皮肠粉</t>
+          <t>果园脆皮烧鸡整只配可乐 2 人份</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>戴记特色腐皮肠粉</t>
+          <t>果园脆皮烧鸡整只配可乐 2人份</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>25</v>
+        <v>108.9</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>潮汕</t>
+          <t>粤菜</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>白肉</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>蒸</t>
+          <t>油炸</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="I33" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="n">
@@ -2169,45 +2165,45 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>d_070_014</t>
+          <t>d_132_052</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>隆凤烧鸡 1 只+毛豆+花生</t>
+          <t>卤蛋</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>隆凤烧鸡1只+毛豆+花生</t>
+          <t>卤蛋</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>93.8</v>
+        <v>3</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>粤菜</t>
+          <t>小吃</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>白肉</t>
+          <t>蛋</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>烤</t>
+          <t>煮</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I34" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J34" t="n">
-        <v>125</v>
+        <v>5</v>
       </c>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="n">
@@ -2219,21 +2215,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>d_091_051</t>
+          <t>d_106_065</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>双肉肠粉</t>
+          <t>枸杞叶（加粥里）</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>双肉肠粉</t>
+          <t>枸杞叶</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>10.8</v>
+        <v>2.9</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -2242,28 +2238,24 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>纯素</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>蒸</t>
+          <t>煮</t>
         </is>
       </c>
       <c r="H35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I35" t="n">
-        <v>0.05</v>
+        <v>0.95</v>
       </c>
       <c r="J35" t="n">
-        <v>16</v>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K35" t="inlineStr"/>
       <c r="L35" t="n">
         <v>0</v>
       </c>
@@ -2273,53 +2265,49 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>d_042_002</t>
+          <t>d_087_064</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>牛肉牛丸汤粿条</t>
+          <t>肉沫（直接加粉里）</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>牛肉牛丸汤粿条</t>
+          <t>肉沫</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>28</v>
+        <v>13.8</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>潮汕</t>
+          <t>湘菜</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>红肉</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>煮</t>
+          <t>炒</t>
         </is>
       </c>
       <c r="H36" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I36" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="J36" t="n">
-        <v>25</v>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>15</v>
+      </c>
+      <c r="K36" t="inlineStr"/>
       <c r="L36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr"/>
@@ -2327,47 +2315,51 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>d_127_051</t>
+          <t>d_046_058</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>蔬果汁柚子包</t>
+          <t>芝士牛肉汉堡套餐</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>蔬果汁柚子包</t>
+          <t>芝士牛肉汉堡套餐</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>29</v>
+        <v>39.9</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>粤菜</t>
+          <t>西式</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>红肉</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>蒸</t>
+          <t>烤</t>
         </is>
       </c>
       <c r="H37" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I37" t="n">
         <v>0.1</v>
       </c>
       <c r="J37" t="n">
-        <v>6</v>
-      </c>
-      <c r="K37" t="inlineStr"/>
+        <v>25</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="L37" t="n">
         <v>0</v>
       </c>
@@ -2377,53 +2369,49 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>d_136_007</t>
+          <t>d_066_024</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>黄焖牛蛙➕自选配菜 2 个➕米饭</t>
+          <t>乌苏啤酒 500ml</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>黄焖牛蛙配菜套餐</t>
+          <t>乌苏啤酒 500ml</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>34.9</v>
+        <v>10</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>快餐</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>白肉</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>炖</t>
+          <t>生</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="I38" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="J38" t="n">
-        <v>30</v>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K38" t="inlineStr"/>
       <c r="L38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr"/>
@@ -2431,25 +2419,25 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>d_002_006</t>
+          <t>d_106_005</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>靓靓家凉面（大份）</t>
+          <t>皮蛋瘦肉砂锅粥</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>靓靓家凉面</t>
+          <t>皮蛋瘦肉砂锅粥</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>22</v>
+        <v>18.8</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>小吃</t>
+          <t>粤菜</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -2459,21 +2447,25 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>凉拌</t>
+          <t>煮</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I39" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="J39" t="n">
-        <v>15</v>
-      </c>
-      <c r="K39" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="L39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr"/>
@@ -2481,17 +2473,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>d_120_031</t>
+          <t>d_026_041</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>双蛋瘦肉肠</t>
+          <t>炭烤茄子#蒜蓉与炭火的碰撞</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>双蛋瘦肉肠粉</t>
+          <t>炭烤茄子</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -2499,35 +2491,31 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>粤菜</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>纯素</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>蒸</t>
+          <t>烤</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I40" t="n">
-        <v>0.05</v>
+        <v>0.9</v>
       </c>
       <c r="J40" t="n">
-        <v>22</v>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K40" t="inlineStr"/>
       <c r="L40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr"/>
@@ -2535,25 +2523,25 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>d_127_022</t>
+          <t>d_024_017</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>广式云吞面</t>
+          <t>酸辣笋尖米线</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>广式云吞面</t>
+          <t>酸辣笋尖米线</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>29</v>
+        <v>19.9</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>粤菜</t>
+          <t>小吃</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2567,13 +2555,13 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I41" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J41" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="K41" t="inlineStr">
         <is>
@@ -2581,7 +2569,7 @@
         </is>
       </c>
       <c r="L41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr"/>
@@ -2589,49 +2577,53 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>d_021_008</t>
+          <t>d_120_039</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>腐竹烧牛腩</t>
+          <t>虾仁滑蛋肠粉</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>腐竹烧牛腩</t>
+          <t>虾仁滑蛋肠粉</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>25.8</v>
+        <v>16.2</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>湘菜</t>
+          <t>粤菜</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>红肉</t>
+          <t>主食</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>炖</t>
+          <t>蒸</t>
         </is>
       </c>
       <c r="H42" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I42" t="n">
-        <v>0.15</v>
+        <v>0.05</v>
       </c>
       <c r="J42" t="n">
-        <v>28</v>
-      </c>
-      <c r="K42" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="L42" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr"/>
@@ -2639,45 +2631,45 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>d_112_002</t>
+          <t>d_025_011</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>火腿肠</t>
+          <t>花甲+脆皮肠+娃娃菜＋金针菇+粉/面</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>火腿肠粉</t>
+          <t>花甲+脆皮肠+娃娃菜+金针菇+粉/面</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>12</v>
+        <v>27.9</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>粤菜</t>
+          <t>小吃</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>海鲜</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>蒸</t>
+          <t>煮</t>
         </is>
       </c>
       <c r="H43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I43" t="n">
-        <v>0.05</v>
+        <v>0.25</v>
       </c>
       <c r="J43" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="K43" t="inlineStr">
         <is>
@@ -2693,49 +2685,49 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>d_064_028</t>
+          <t>d_114_026</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>特大蟹（1 只）</t>
+          <t>辣椒酱</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>特大蟹</t>
+          <t>辣椒酱</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>238</v>
+        <v>18</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>粤菜</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>海鲜</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>煮</t>
+          <t>凉拌</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="J44" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr"/>
@@ -2743,30 +2735,30 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>d_049_074</t>
+          <t>d_109_042</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>白水煮蛋(一个)</t>
+          <t>海鲜汤米粉</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>白水煮蛋</t>
+          <t>海鲜汤米粉</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>3.5</v>
+        <v>20.8</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>小吃</t>
+          <t>潮汕</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>蛋</t>
+          <t>主食</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2775,15 +2767,19 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="J45" t="n">
-        <v>6</v>
-      </c>
-      <c r="K45" t="inlineStr"/>
+        <v>15</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="L45" t="n">
         <v>0</v>
       </c>
@@ -2793,49 +2789,53 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>d_039_074</t>
+          <t>d_196_001</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>生态藕尖</t>
+          <t>超值两荤两素任你选【贼阔气】+2 荤 2 素</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>生态藕尖</t>
+          <t>超值两荤两素套餐</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>18.8</v>
+        <v>23</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>小吃</t>
+          <t>东北</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>纯素</t>
+          <t>红肉</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>凉拌</t>
+          <t>炒</t>
         </is>
       </c>
       <c r="H46" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I46" t="n">
-        <v>0.9</v>
+        <v>0.4</v>
       </c>
       <c r="J46" t="n">
-        <v>3</v>
-      </c>
-      <c r="K46" t="inlineStr"/>
+        <v>25</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
       <c r="L46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr"/>
@@ -2843,49 +2843,49 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>d_020_039</t>
+          <t>d_083_028</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>辣椒</t>
+          <t>吉士蛋元气堡</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>辣椒</t>
+          <t>吉士蛋元气堡</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>16.7</v>
+        <v>7.9</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>东北</t>
+          <t>西式</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>纯素</t>
+          <t>蛋</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>烤</t>
+          <t>煎</t>
         </is>
       </c>
       <c r="H47" t="n">
         <v>3</v>
       </c>
       <c r="I47" t="n">
-        <v>0.9</v>
+        <v>0.05</v>
       </c>
       <c r="J47" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr"/>
@@ -2893,30 +2893,30 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>d_027_058</t>
+          <t>d_012_066</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>招牌双拼（半只原味+半只香辣）</t>
+          <t>【鸿运马年】佳人双对（110 串）</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>招牌双拼 半只原味+半只香辣</t>
+          <t>佳人双对 110 串</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>78.90000000000001</v>
+        <v>144.9</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>粤菜</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>白肉</t>
+          <t>红肉</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2925,13 +2925,13 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I48" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="J48" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="n">
@@ -2943,25 +2943,25 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>d_120_069</t>
+          <t>d_145_011</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>鲜奶小馒头【加赠炼奶】</t>
+          <t>☀️封神烧椒牛腩菠菜面（不可免辣）</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>鲜奶小馒头</t>
+          <t>封神烧椒牛腩菠菜面</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>8.800000000000001</v>
+        <v>37</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>小吃</t>
+          <t>西北</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
@@ -2971,21 +2971,25 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>蒸</t>
+          <t>煮</t>
         </is>
       </c>
       <c r="H49" t="n">
+        <v>4</v>
+      </c>
+      <c r="I49" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J49" t="n">
+        <v>20</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L49" t="n">
         <v>2</v>
-      </c>
-      <c r="I49" t="n">
-        <v>0</v>
-      </c>
-      <c r="J49" t="n">
-        <v>5</v>
-      </c>
-      <c r="K49" t="inlineStr"/>
-      <c r="L49" t="n">
-        <v>0</v>
       </c>
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr"/>
@@ -2993,49 +2997,53 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>d_049_044</t>
+          <t>d_173_034</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>韭菜鸡蛋大包子(1 个)</t>
+          <t>爆炒腊鸭腿+江西炒米粉套餐</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>韭菜鸡蛋大包子</t>
+          <t>爆炒腊鸭腿+江西炒米粉套餐</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>4.9</v>
+        <v>45.8</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>小吃</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>主食</t>
+          <t>白肉</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>蒸</t>
+          <t>炒</t>
         </is>
       </c>
       <c r="H50" t="n">
+        <v>5</v>
+      </c>
+      <c r="I50" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J50" t="n">
+        <v>30</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="L50" t="n">
         <v>2</v>
-      </c>
-      <c r="I50" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="J50" t="n">
-        <v>5</v>
-      </c>
-      <c r="K50" t="inlineStr"/>
-      <c r="L50" t="n">
-        <v>0</v>
       </c>
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr"/>
@@ -3043,30 +3051,30 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>d_014_040</t>
+          <t>d_033_035</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>鲜雪花牛肉</t>
+          <t>化骨绵掌（鸭掌）10 串</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>鲜雪花牛肉</t>
+          <t>鸭掌 10 串</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>4.9</v>
+        <v>18</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>小吃</t>
+          <t>其他</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>红肉</t>
+          <t>白肉</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3075,17 +3083,17 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I51" t="n">
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr"/>
@@ -3138,7 +3146,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7256</v>
+        <v>11123</v>
       </c>
     </row>
     <row r="4">

</xml_diff>